<commit_message>
updated ERP checking and fatal error handling
</commit_message>
<xml_diff>
--- a/static/static_ERPTs.xlsx
+++ b/static/static_ERPTs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55586\Desktop\tools\access tool\access-tool-migration\static\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\17475\Downloads\RTR2HEM_20231117\RTR2HEM\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8262F89C-E8F1-4F2D-A26A-1F121D11D76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888415E9-A689-4E57-A524-94B6B9867592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5505" yWindow="5040" windowWidth="24825" windowHeight="14940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>EMISSION_RELEASE_POINT_TYPE</t>
   </si>
@@ -76,9 +76,6 @@
     <t>7</t>
   </si>
   <si>
-    <t>FUGITIVE AREA (RESERVED FOR HISTORICAL DATA)</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -94,19 +91,10 @@
     <t>N (Line)</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>FUGITIVE THREE-DIMENSIONAL</t>
   </si>
   <si>
     <t>V (Volume)</t>
-  </si>
-  <si>
-    <t>99</t>
-  </si>
-  <si>
-    <t>UNKNOWN</t>
   </si>
 </sst>
 </file>
@@ -126,11 +114,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -195,13 +185,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" customWidth="1"/>
@@ -593,22 +586,22 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>5</v>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>8</v>
@@ -616,35 +609,13 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>